<commit_message>
PQ50: final review round 2 - vendor spec wording, table precision
Every equation and calculation block of the English AN was recomputed;
none disagreed. The figures not viewed in round 1 were checked.

- Vendor spec: NP1 "15 Ts" -> "15 T"; note 32 now depends on the
  variant (single transformer: the reference construction sets item 3-2).
- Tables: lambda 0.556, n 6.013, phase margin 49.6 deg, lN 100.5 mm in
  the first leakage estimate, fo 44.8 kHz in the spec summary.
- HISTORY row 77.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/PQ50/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x1.xlsx
+++ b/PQ50/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x1.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>15 Ts</t>
+          <t>15 T</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -957,7 +957,7 @@
     <row r="32" ht="14" customHeight="1">
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>Core, bobbin, wire and winding arrangement are the supplier’s choice, provided sections 3 and 5 are met.</t>
+          <t>The core, coil former and winding arrangement of the reference design set item 3-2. Another construction is acceptable only when sections 3 and 5 are met and the first samples are approved.</t>
         </is>
       </c>
     </row>

</xml_diff>